<commit_message>
fix: resolve missing sold dates for 寿臣山15号 on HKP API and rebuild web database
</commit_message>
<xml_diff>
--- a/files/港岛-寿臣山-寿臣山15号.xlsx
+++ b/files/港岛-寿臣山-寿臣山15号.xlsx
@@ -609,7 +609,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -755,7 +755,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2024-10-31</t>
         </is>
       </c>
       <c r="H4" s="5" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2024-08-11</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
@@ -847,7 +847,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2024-03-04</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
@@ -893,7 +893,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
@@ -939,7 +939,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2022-07-21</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2024-05-21</t>
         </is>
       </c>
       <c r="H9" s="5" t="n">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="H10" s="5" t="n">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="H11" s="5" t="n">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2022-08-07</t>
         </is>
       </c>
       <c r="H12" s="5" t="n">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2024-07-29</t>
         </is>
       </c>
       <c r="H13" s="5" t="n">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="H14" s="5" t="n">
@@ -1534,7 +1534,7 @@
         <is>
           <t>2号屋
 12073呎 (4+房)
-(已售)
+(24年-10月)
 $8.45亿
 $69,991/呎</t>
         </is>
@@ -1543,7 +1543,7 @@
         <is>
           <t>3号屋
 9694呎 (4+房)
-(已售)
+(24年-08月)
 $7.17亿
 $74,000/呎</t>
         </is>
@@ -1552,7 +1552,7 @@
         <is>
           <t>5号屋
 6695呎 (4+房)
-(已售)
+(24年-03月)
 $4.98亿
 $74,400/呎</t>
         </is>
@@ -1561,7 +1561,7 @@
         <is>
           <t>6号屋
 9550呎 (4+房)
-(已售)
+(25年-10月)
 $5.79亿
 $60,623/呎</t>
         </is>
@@ -1570,7 +1570,7 @@
         <is>
           <t>7号屋
 8032呎 (4+房)
-(已售)
+(22年-07月)
 $8.70亿
 $108,347/呎</t>
         </is>
@@ -1586,7 +1586,7 @@
         <is>
           <t>8号屋
 2746呎 (4+房)
-(已售)
+(24年-05月)
 $2.60亿
 $94,670/呎</t>
         </is>
@@ -1595,7 +1595,7 @@
         <is>
           <t>9号屋
 3727呎 (4+房)
-(已售)
+(26年-01月)
 $2.25亿
 $60,263/呎</t>
         </is>
@@ -1604,7 +1604,7 @@
         <is>
           <t>10号屋
 4853呎 (4+房)
-(已售)
+(26年-01月)
 $2.92亿
 $60,264/呎</t>
         </is>
@@ -1613,7 +1613,7 @@
         <is>
           <t>11号屋
 4759呎 (4+房)
-(已售)
+(22年-08月)
 $4.35亿
 $91,406/呎</t>
         </is>
@@ -1622,7 +1622,7 @@
         <is>
           <t>12号屋
 4696呎 (4+房)
-(已售)
+(24年-07月)
 $3.20亿
 $68,177/呎</t>
         </is>
@@ -1631,7 +1631,7 @@
         <is>
           <t>15号屋
 4696呎 (4+房)
-(已售)
+(26年-01月)
 $2.90亿
 $61,725/呎</t>
         </is>

</xml_diff>